<commit_message>
docs(ux): simplificar informe de hallazgos Fase 2 y generar PDF
Reescribe el informe con redacción directa y resumen al inicio, reduce la
nomenclatura interna y deja la planificación por sprint como
recomendación. Registra la fecha de las sesiones y marca como probable la
causa del problema de legibilidad en marketing.

Alinea los identificadores de la hoja Hallazgos con el informe y agrega
la versión en PDF.
</commit_message>
<xml_diff>
--- a/docs/pruebas-usabilidad/Registro_sesiones_usabilidad_Fase_2.xlsx
+++ b/docs/pruebas-usabilidad/Registro_sesiones_usabilidad_Fase_2.xlsx
@@ -10573,7 +10573,7 @@
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>H2-01</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B6" s="26" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>Acceso de venta en la navegación con vocabulario del usuario; «Vender» como acción principal de la tarjeta; panel de venta visible antes del primer producto. Sprint 9</t>
+          <t>Acceso de venta en la navegación con vocabulario del usuario; «Vender» como acción principal de la tarjeta; panel de venta visible antes del primer producto. Sprint recomendado: 9</t>
         </is>
       </c>
       <c r="I6" s="26" t="inlineStr">
@@ -10641,7 +10641,7 @@
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>H2-02</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>Opciones de proyecto y formato ilegibles sin pasar el cursor (selectores sin fondo explícito de opción)</t>
+          <t>Opciones de proyecto y formato ilegibles sin pasar el cursor (causa probable: selectores sin fondo explícito de opción; reproducir antes de corregir)</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
@@ -10676,7 +10676,7 @@
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
-          <t>Fondo y texto explícitos en las opciones de los selectores de marketing y proveedores; contraste AA. Sprint 9</t>
+          <t>Fondo y texto explícitos en las opciones de los selectores de marketing y proveedores; contraste AA. Sprint recomendado: 9</t>
         </is>
       </c>
       <c r="I7" s="26" t="inlineStr">
@@ -10709,7 +10709,7 @@
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>H2-03</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B8" s="26" t="inlineStr">
@@ -10744,7 +10744,7 @@
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>Confirmación visible junto a «Realizar venta»; rótulo de existencias en lenguaje llano. Sprint 10</t>
+          <t>Confirmación visible junto a «Realizar venta»; rótulo de existencias en lenguaje llano. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I8" s="26" t="inlineStr">
@@ -10777,7 +10777,7 @@
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>H2-04</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="H9" s="26" t="inlineStr">
         <is>
-          <t>«Guardar» como acción de mayor peso; confirmación al cancelar con datos. Sprint 10</t>
+          <t>«Guardar» como acción de mayor peso; confirmación al cancelar con datos. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I9" s="26" t="inlineStr">
@@ -10845,7 +10845,7 @@
     <row r="10" ht="52" customHeight="1">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>H2-05</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B10" s="26" t="inlineStr">
@@ -10880,7 +10880,7 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>«Nueva publicación» como acción de mayor jerarquía de la vista. Sprint 10</t>
+          <t>«Nueva publicación» como acción de mayor jerarquía de la vista. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I10" s="26" t="inlineStr">
@@ -10913,7 +10913,7 @@
     <row r="11" ht="52" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>H2-06</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
@@ -10948,7 +10948,7 @@
       </c>
       <c r="H11" s="26" t="inlineStr">
         <is>
-          <t>Acción visible para abrir la ficha desde la tarjeta; sección traducida; acceso desde Proveedores. Sprint 10</t>
+          <t>Acción visible para abrir la ficha desde la tarjeta; sección traducida; acceso desde Proveedores. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I11" s="26" t="inlineStr">
@@ -10981,7 +10981,7 @@
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>H2-07</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B12" s="26" t="inlineStr">
@@ -11016,7 +11016,7 @@
       </c>
       <c r="H12" s="26" t="inlineStr">
         <is>
-          <t>Acceso directo a «Nuevo producto» desde el dashboard; navegación que mencione productos. Sprint 10</t>
+          <t>Acceso directo a «Nuevo producto» desde el dashboard; navegación que mencione productos. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I12" s="26" t="inlineStr">
@@ -11049,7 +11049,7 @@
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>H2-08</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
@@ -11084,7 +11084,7 @@
       </c>
       <c r="H13" s="26" t="inlineStr">
         <is>
-          <t>Rótulos visibles en los filtros de publicaciones. Sprint 10</t>
+          <t>Rótulos visibles en los filtros de publicaciones. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I13" s="26" t="inlineStr">
@@ -11117,7 +11117,7 @@
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>H2-09</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B14" s="26" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="H14" s="26" t="inlineStr">
         <is>
-          <t>Auditoría de contraste AA de los textos secundarios de la tarjeta. Sprint 10</t>
+          <t>Auditoría de contraste AA de los textos secundarios de la tarjeta. Sprint recomendado: 10</t>
         </is>
       </c>
       <c r="I14" s="26" t="inlineStr">
@@ -11185,7 +11185,7 @@
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="B15" s="26" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
-          <t>Corregir manejo de zona horaria de scheduled_for (timestamp sin zona + node-pg en UTC). Bug, Sprint 9</t>
+          <t>Corregir manejo de zona horaria de scheduled_for (timestamp sin zona + node-pg en UTC). Bug, Sprint recomendado: 9</t>
         </is>
       </c>
       <c r="I15" s="26" t="inlineStr">

</xml_diff>